<commit_message>
feat: Subindo Apache POI + JDBC finalizado
</commit_message>
<xml_diff>
--- a/api-etl-java/turismo-rio-de-janeiro.xlsx
+++ b/api-etl-java/turismo-rio-de-janeiro.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9acbaa33c33b352b/Área de Trabalho/SPTECH/2 Semestre/PI/TourTech/api-etl-java/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{20D251BD-B3CA-4287-934B-61B5EA2B84AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DAE6C8C-AF38-4B5A-AFF4-465F538EA3F2}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="8_{20D251BD-B3CA-4287-934B-61B5EA2B84AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB318045-F883-47EB-97C6-97AA04DC9D3D}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0A7E5AAC-7087-4E10-9ED1-14D0BB1A0403}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0A7E5AAC-7087-4E10-9ED1-14D0BB1A0403}"/>
   </bookViews>
   <sheets>
     <sheet name="Turismo Internacional por País" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
   <si>
     <t>País de Origem</t>
   </si>
@@ -78,72 +78,6 @@
     <t>DEZ</t>
   </si>
   <si>
-    <t>TOTAL</t>
-  </si>
-  <si>
-    <t>1. Argentina</t>
-  </si>
-  <si>
-    <t>2. Chile</t>
-  </si>
-  <si>
-    <t>3. Estados Unidos</t>
-  </si>
-  <si>
-    <t>4. França</t>
-  </si>
-  <si>
-    <t>5. Uruguai</t>
-  </si>
-  <si>
-    <t>6. Colômbia</t>
-  </si>
-  <si>
-    <t>7. Peru</t>
-  </si>
-  <si>
-    <t>8. Portugal</t>
-  </si>
-  <si>
-    <t>9. México</t>
-  </si>
-  <si>
-    <t>10. Reino Unido</t>
-  </si>
-  <si>
-    <t>11. Alemanha</t>
-  </si>
-  <si>
-    <t>12. Espanha</t>
-  </si>
-  <si>
-    <t>13. Itália</t>
-  </si>
-  <si>
-    <t>14. Canadá</t>
-  </si>
-  <si>
-    <t>15. Equador</t>
-  </si>
-  <si>
-    <t>16. Paraguai</t>
-  </si>
-  <si>
-    <t>17. Países Baixos</t>
-  </si>
-  <si>
-    <t>18. China</t>
-  </si>
-  <si>
-    <t>19. Suíça</t>
-  </si>
-  <si>
-    <t>20. Coreia do Sul</t>
-  </si>
-  <si>
-    <t>21. Outros</t>
-  </si>
-  <si>
     <t>Estado de Origem</t>
   </si>
   <si>
@@ -229,6 +163,66 @@
   </si>
   <si>
     <t>Id</t>
+  </si>
+  <si>
+    <t>Argentina</t>
+  </si>
+  <si>
+    <t>Chile</t>
+  </si>
+  <si>
+    <t>Estados Unidos</t>
+  </si>
+  <si>
+    <t>França</t>
+  </si>
+  <si>
+    <t>Uruguai</t>
+  </si>
+  <si>
+    <t>Colômbia</t>
+  </si>
+  <si>
+    <t>Peru</t>
+  </si>
+  <si>
+    <t>Portugal</t>
+  </si>
+  <si>
+    <t>México</t>
+  </si>
+  <si>
+    <t>Reino Unido</t>
+  </si>
+  <si>
+    <t>Espanha</t>
+  </si>
+  <si>
+    <t>Alemanha</t>
+  </si>
+  <si>
+    <t>Itália</t>
+  </si>
+  <si>
+    <t>Canadá</t>
+  </si>
+  <si>
+    <t>Equador</t>
+  </si>
+  <si>
+    <t>Paraguai</t>
+  </si>
+  <si>
+    <t>Países Baixos</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>Suíça</t>
+  </si>
+  <si>
+    <t>Coreia do Sul</t>
   </si>
 </sst>
 </file>
@@ -601,978 +595,934 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{062DEA4F-A5BC-4B7D-8A9B-D5676DAD4358}">
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="1">
+        <v>77954</v>
+      </c>
+      <c r="D2" s="1">
+        <v>67774</v>
+      </c>
+      <c r="E2" s="1">
+        <v>67626</v>
+      </c>
+      <c r="F2" s="1">
+        <v>28101</v>
+      </c>
+      <c r="G2" s="1">
+        <v>20260</v>
+      </c>
+      <c r="H2" s="1">
+        <v>17969</v>
+      </c>
+      <c r="I2" s="1">
+        <v>27361</v>
+      </c>
+      <c r="J2" s="1">
+        <v>21191</v>
+      </c>
+      <c r="K2" s="1">
+        <v>25857</v>
+      </c>
+      <c r="L2" s="1">
+        <v>33047</v>
+      </c>
+      <c r="M2" s="1">
+        <v>32178</v>
+      </c>
+      <c r="N2" s="1">
+        <v>48719</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="1">
+        <v>25478</v>
+      </c>
+      <c r="D3" s="1">
+        <v>45358</v>
+      </c>
+      <c r="E3" s="1">
+        <v>30363</v>
+      </c>
+      <c r="F3" s="1">
+        <v>13784</v>
+      </c>
+      <c r="G3" s="1">
+        <v>8026</v>
+      </c>
+      <c r="H3" s="1">
+        <v>9097</v>
+      </c>
+      <c r="I3" s="1">
+        <v>8582</v>
+      </c>
+      <c r="J3" s="1">
+        <v>8791</v>
+      </c>
+      <c r="K3" s="1">
+        <v>16840</v>
+      </c>
+      <c r="L3" s="1">
+        <v>21407</v>
+      </c>
+      <c r="M3" s="1">
+        <v>22179</v>
+      </c>
+      <c r="N3" s="1">
+        <v>29560</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="1">
+        <v>8140</v>
+      </c>
+      <c r="D4" s="1">
+        <v>19138</v>
+      </c>
+      <c r="E4" s="1">
+        <v>19040</v>
+      </c>
+      <c r="F4" s="1">
+        <v>10122</v>
+      </c>
+      <c r="G4" s="1">
+        <v>13745</v>
+      </c>
+      <c r="H4" s="1">
+        <v>12991</v>
+      </c>
+      <c r="I4" s="1">
+        <v>13740</v>
+      </c>
+      <c r="J4" s="1">
+        <v>14352</v>
+      </c>
+      <c r="K4" s="1">
+        <v>15296</v>
+      </c>
+      <c r="L4" s="1">
+        <v>14779</v>
+      </c>
+      <c r="M4" s="1">
+        <v>19482</v>
+      </c>
+      <c r="N4" s="1">
+        <v>24775</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="1">
+        <v>4781</v>
+      </c>
+      <c r="D5" s="1">
+        <v>11432</v>
+      </c>
+      <c r="E5" s="1">
+        <v>7683</v>
+      </c>
+      <c r="F5" s="1">
+        <v>3825</v>
+      </c>
+      <c r="G5" s="1">
+        <v>3173</v>
+      </c>
+      <c r="H5" s="1">
+        <v>1927</v>
+      </c>
+      <c r="I5" s="1">
+        <v>3891</v>
+      </c>
+      <c r="J5" s="1">
+        <v>7406</v>
+      </c>
+      <c r="K5" s="1">
+        <v>6428</v>
+      </c>
+      <c r="L5" s="1">
+        <v>8734</v>
+      </c>
+      <c r="M5" s="1">
+        <v>5474</v>
+      </c>
+      <c r="N5" s="1">
+        <v>5361</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="1">
+        <v>8614</v>
+      </c>
+      <c r="D6" s="1">
+        <v>8288</v>
+      </c>
+      <c r="E6" s="1">
+        <v>10849</v>
+      </c>
+      <c r="F6" s="1">
+        <v>3173</v>
+      </c>
+      <c r="G6" s="1">
+        <v>2915</v>
+      </c>
+      <c r="H6" s="1">
+        <v>2405</v>
+      </c>
+      <c r="I6" s="1">
+        <v>4023</v>
+      </c>
+      <c r="J6" s="1">
+        <v>3813</v>
+      </c>
+      <c r="K6" s="1">
+        <v>6468</v>
+      </c>
+      <c r="L6" s="1">
+        <v>7910</v>
+      </c>
+      <c r="M6" s="1">
+        <v>4638</v>
+      </c>
+      <c r="N6" s="1">
+        <v>6611</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="1">
+        <v>2725</v>
+      </c>
+      <c r="D7" s="1">
+        <v>2405</v>
+      </c>
+      <c r="E7" s="1">
+        <v>4588</v>
+      </c>
+      <c r="F7" s="1">
+        <v>2817</v>
+      </c>
+      <c r="G7" s="1">
+        <v>3410</v>
+      </c>
+      <c r="H7" s="1">
+        <v>3769</v>
+      </c>
+      <c r="I7" s="1">
+        <v>2890</v>
+      </c>
+      <c r="J7" s="1">
+        <v>3259</v>
+      </c>
+      <c r="K7" s="1">
+        <v>3373</v>
+      </c>
+      <c r="L7" s="1">
+        <v>5372</v>
+      </c>
+      <c r="M7" s="1">
+        <v>4465</v>
+      </c>
+      <c r="N7" s="1">
+        <v>4747</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="1">
+        <v>2322</v>
+      </c>
+      <c r="D8" s="1">
+        <v>4159</v>
+      </c>
+      <c r="E8" s="1">
+        <v>4587</v>
+      </c>
+      <c r="F8" s="1">
+        <v>2674</v>
+      </c>
+      <c r="G8" s="1">
+        <v>3032</v>
+      </c>
+      <c r="H8" s="1">
+        <v>2421</v>
+      </c>
+      <c r="I8" s="1">
+        <v>2404</v>
+      </c>
+      <c r="J8" s="1">
+        <v>3854</v>
+      </c>
+      <c r="K8" s="1">
+        <v>3150</v>
+      </c>
+      <c r="L8" s="1">
+        <v>4322</v>
+      </c>
+      <c r="M8" s="1">
+        <v>3940</v>
+      </c>
+      <c r="N8" s="1">
+        <v>3751</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="1">
+        <v>2273</v>
+      </c>
+      <c r="D9" s="1">
+        <v>4684</v>
+      </c>
+      <c r="E9" s="1">
+        <v>4746</v>
+      </c>
+      <c r="F9" s="1">
+        <v>1739</v>
+      </c>
+      <c r="G9" s="1">
+        <v>1275</v>
+      </c>
+      <c r="H9" s="1">
+        <v>1194</v>
+      </c>
+      <c r="I9" s="1">
+        <v>1483</v>
+      </c>
+      <c r="J9" s="1">
+        <v>2134</v>
+      </c>
+      <c r="K9" s="1">
+        <v>2316</v>
+      </c>
+      <c r="L9" s="1">
+        <v>2499</v>
+      </c>
+      <c r="M9" s="1">
+        <v>3710</v>
+      </c>
+      <c r="N9" s="1">
+        <v>4393</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1502</v>
+      </c>
+      <c r="D10" s="1">
+        <v>2448</v>
+      </c>
+      <c r="E10" s="1">
+        <v>2720</v>
+      </c>
+      <c r="F10" s="1">
+        <v>2095</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1797</v>
+      </c>
+      <c r="H10" s="1">
+        <v>1923</v>
+      </c>
+      <c r="I10" s="1">
+        <v>2185</v>
+      </c>
+      <c r="J10" s="1">
+        <v>2705</v>
+      </c>
+      <c r="K10" s="1">
+        <v>2393</v>
+      </c>
+      <c r="L10" s="1">
+        <v>2313</v>
+      </c>
+      <c r="M10" s="1">
+        <v>2632</v>
+      </c>
+      <c r="N10" s="1">
+        <v>2482</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="1">
+        <v>2080</v>
+      </c>
+      <c r="D11" s="1">
+        <v>3337</v>
+      </c>
+      <c r="E11" s="1">
+        <v>2797</v>
+      </c>
+      <c r="F11" s="1">
+        <v>1455</v>
+      </c>
+      <c r="G11" s="1">
+        <v>1367</v>
+      </c>
+      <c r="H11" s="1">
+        <v>1162</v>
+      </c>
+      <c r="I11" s="1">
+        <v>1385</v>
+      </c>
+      <c r="J11" s="1">
+        <v>1527</v>
+      </c>
+      <c r="K11" s="1">
+        <v>1937</v>
+      </c>
+      <c r="L11" s="1">
+        <v>1986</v>
+      </c>
+      <c r="M11" s="1">
+        <v>2243</v>
+      </c>
+      <c r="N11" s="1">
+        <v>2669</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="1">
+        <v>1256</v>
+      </c>
+      <c r="D12" s="1">
+        <v>3305</v>
+      </c>
+      <c r="E12" s="1">
+        <v>3322</v>
+      </c>
+      <c r="F12" s="1">
+        <v>1487</v>
+      </c>
+      <c r="G12" s="1">
+        <v>1147</v>
+      </c>
+      <c r="H12">
+        <v>783</v>
+      </c>
+      <c r="I12" s="1">
+        <v>1568</v>
+      </c>
+      <c r="J12" s="1">
+        <v>1746</v>
+      </c>
+      <c r="K12" s="1">
+        <v>1767</v>
+      </c>
+      <c r="L12" s="1">
+        <v>2339</v>
+      </c>
+      <c r="M12" s="1">
+        <v>2340</v>
+      </c>
+      <c r="N12" s="1">
+        <v>2286</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" s="1">
+        <v>1389</v>
+      </c>
+      <c r="D13" s="1">
+        <v>2018</v>
+      </c>
+      <c r="E13" s="1">
+        <v>2096</v>
+      </c>
+      <c r="F13" s="1">
+        <v>1193</v>
+      </c>
+      <c r="G13" s="1">
+        <v>1010</v>
+      </c>
+      <c r="H13">
+        <v>755</v>
+      </c>
+      <c r="I13" s="1">
+        <v>1265</v>
+      </c>
+      <c r="J13" s="1">
+        <v>1852</v>
+      </c>
+      <c r="K13" s="1">
+        <v>1078</v>
+      </c>
+      <c r="L13" s="1">
+        <v>1120</v>
+      </c>
+      <c r="M13" s="1">
+        <v>1549</v>
+      </c>
+      <c r="N13" s="1">
+        <v>2037</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="B14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14">
+        <v>764</v>
+      </c>
+      <c r="D14" s="1">
+        <v>2382</v>
+      </c>
+      <c r="E14" s="1">
+        <v>1828</v>
+      </c>
+      <c r="F14" s="1">
+        <v>1019</v>
+      </c>
+      <c r="G14">
+        <v>559</v>
+      </c>
+      <c r="H14">
+        <v>580</v>
+      </c>
+      <c r="I14">
+        <v>814</v>
+      </c>
+      <c r="J14" s="1">
+        <v>2399</v>
+      </c>
+      <c r="K14" s="1">
+        <v>1252</v>
+      </c>
+      <c r="L14" s="1">
+        <v>1103</v>
+      </c>
+      <c r="M14" s="1">
+        <v>1804</v>
+      </c>
+      <c r="N14" s="1">
+        <v>2602</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15">
         <v>14</v>
       </c>
-      <c r="B2" s="1">
-        <v>77954</v>
-      </c>
-      <c r="C2" s="1">
-        <v>67774</v>
-      </c>
-      <c r="D2" s="1">
-        <v>67626</v>
-      </c>
-      <c r="E2" s="1">
-        <v>28101</v>
-      </c>
-      <c r="F2" s="1">
-        <v>20260</v>
-      </c>
-      <c r="G2" s="1">
-        <v>17969</v>
-      </c>
-      <c r="H2" s="1">
-        <v>27361</v>
-      </c>
-      <c r="I2" s="1">
-        <v>21191</v>
-      </c>
-      <c r="J2" s="1">
-        <v>25857</v>
-      </c>
-      <c r="K2" s="1">
-        <v>33047</v>
-      </c>
-      <c r="L2" s="1">
-        <v>32178</v>
-      </c>
-      <c r="M2" s="1">
-        <v>48719</v>
-      </c>
-      <c r="N2" s="1">
-        <v>468037</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="1">
+        <v>2322</v>
+      </c>
+      <c r="D15" s="1">
+        <v>2776</v>
+      </c>
+      <c r="E15" s="1">
+        <v>2537</v>
+      </c>
+      <c r="F15">
+        <v>975</v>
+      </c>
+      <c r="G15">
+        <v>709</v>
+      </c>
+      <c r="H15">
+        <v>470</v>
+      </c>
+      <c r="I15">
+        <v>685</v>
+      </c>
+      <c r="J15">
+        <v>794</v>
+      </c>
+      <c r="K15">
+        <v>717</v>
+      </c>
+      <c r="L15">
+        <v>929</v>
+      </c>
+      <c r="M15" s="1">
+        <v>1338</v>
+      </c>
+      <c r="N15" s="1">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16">
         <v>15</v>
       </c>
-      <c r="B3" s="1">
-        <v>25478</v>
-      </c>
-      <c r="C3" s="1">
-        <v>45358</v>
-      </c>
-      <c r="D3" s="1">
-        <v>30363</v>
-      </c>
-      <c r="E3" s="1">
-        <v>13784</v>
-      </c>
-      <c r="F3" s="1">
-        <v>8026</v>
-      </c>
-      <c r="G3" s="1">
-        <v>9097</v>
-      </c>
-      <c r="H3" s="1">
-        <v>8582</v>
-      </c>
-      <c r="I3" s="1">
-        <v>8791</v>
-      </c>
-      <c r="J3" s="1">
-        <v>16840</v>
-      </c>
-      <c r="K3" s="1">
-        <v>21407</v>
-      </c>
-      <c r="L3" s="1">
-        <v>22179</v>
-      </c>
-      <c r="M3" s="1">
-        <v>29560</v>
-      </c>
-      <c r="N3" s="1">
-        <v>239465</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B16" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16">
+        <v>442</v>
+      </c>
+      <c r="D16" s="1">
+        <v>1460</v>
+      </c>
+      <c r="E16" s="1">
+        <v>1530</v>
+      </c>
+      <c r="F16" s="1">
+        <v>1116</v>
+      </c>
+      <c r="G16">
+        <v>652</v>
+      </c>
+      <c r="H16">
+        <v>786</v>
+      </c>
+      <c r="I16">
+        <v>527</v>
+      </c>
+      <c r="J16" s="1">
+        <v>1000</v>
+      </c>
+      <c r="K16" s="1">
+        <v>1453</v>
+      </c>
+      <c r="L16" s="1">
+        <v>1330</v>
+      </c>
+      <c r="M16" s="1">
+        <v>1098</v>
+      </c>
+      <c r="N16" s="1">
+        <v>1057</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>16</v>
       </c>
-      <c r="B4" s="1">
-        <v>8140</v>
-      </c>
-      <c r="C4" s="1">
-        <v>19138</v>
-      </c>
-      <c r="D4" s="1">
-        <v>19040</v>
-      </c>
-      <c r="E4" s="1">
-        <v>10122</v>
-      </c>
-      <c r="F4" s="1">
-        <v>13745</v>
-      </c>
-      <c r="G4" s="1">
-        <v>12991</v>
-      </c>
-      <c r="H4" s="1">
-        <v>13740</v>
-      </c>
-      <c r="I4" s="1">
-        <v>14352</v>
-      </c>
-      <c r="J4" s="1">
-        <v>15296</v>
-      </c>
-      <c r="K4" s="1">
-        <v>14779</v>
-      </c>
-      <c r="L4" s="1">
-        <v>19482</v>
-      </c>
-      <c r="M4" s="1">
-        <v>24775</v>
-      </c>
-      <c r="N4" s="1">
-        <v>185600</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C17" s="1">
+        <v>3933</v>
+      </c>
+      <c r="D17" s="1">
+        <v>2542</v>
+      </c>
+      <c r="E17" s="1">
+        <v>2164</v>
+      </c>
+      <c r="F17">
+        <v>308</v>
+      </c>
+      <c r="G17">
+        <v>483</v>
+      </c>
+      <c r="H17">
+        <v>137</v>
+      </c>
+      <c r="I17">
+        <v>220</v>
+      </c>
+      <c r="J17">
+        <v>233</v>
+      </c>
+      <c r="K17">
+        <v>400</v>
+      </c>
+      <c r="L17">
+        <v>365</v>
+      </c>
+      <c r="M17">
+        <v>498</v>
+      </c>
+      <c r="N17">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>17</v>
       </c>
-      <c r="B5" s="1">
-        <v>4781</v>
-      </c>
-      <c r="C5" s="1">
-        <v>11432</v>
-      </c>
-      <c r="D5" s="1">
-        <v>7683</v>
-      </c>
-      <c r="E5" s="1">
-        <v>3825</v>
-      </c>
-      <c r="F5" s="1">
-        <v>3173</v>
-      </c>
-      <c r="G5" s="1">
-        <v>1927</v>
-      </c>
-      <c r="H5" s="1">
-        <v>3891</v>
-      </c>
-      <c r="I5" s="1">
-        <v>7406</v>
-      </c>
-      <c r="J5" s="1">
-        <v>6428</v>
-      </c>
-      <c r="K5" s="1">
-        <v>8734</v>
-      </c>
-      <c r="L5" s="1">
-        <v>5474</v>
-      </c>
-      <c r="M5" s="1">
-        <v>5361</v>
-      </c>
-      <c r="N5" s="1">
-        <v>70115</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B18" t="s">
+        <v>58</v>
+      </c>
+      <c r="C18">
+        <v>714</v>
+      </c>
+      <c r="D18" s="1">
+        <v>1308</v>
+      </c>
+      <c r="E18" s="1">
+        <v>1100</v>
+      </c>
+      <c r="F18">
+        <v>650</v>
+      </c>
+      <c r="G18">
+        <v>560</v>
+      </c>
+      <c r="H18">
+        <v>555</v>
+      </c>
+      <c r="I18">
+        <v>966</v>
+      </c>
+      <c r="J18">
+        <v>931</v>
+      </c>
+      <c r="K18">
+        <v>894</v>
+      </c>
+      <c r="L18" s="1">
+        <v>1049</v>
+      </c>
+      <c r="M18" s="1">
+        <v>1157</v>
+      </c>
+      <c r="N18" s="1">
+        <v>1321</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>18</v>
       </c>
-      <c r="B6" s="1">
-        <v>8614</v>
-      </c>
-      <c r="C6" s="1">
-        <v>8288</v>
-      </c>
-      <c r="D6" s="1">
-        <v>10849</v>
-      </c>
-      <c r="E6" s="1">
-        <v>3173</v>
-      </c>
-      <c r="F6" s="1">
-        <v>2915</v>
-      </c>
-      <c r="G6" s="1">
-        <v>2405</v>
-      </c>
-      <c r="H6" s="1">
-        <v>4023</v>
-      </c>
-      <c r="I6" s="1">
-        <v>3813</v>
-      </c>
-      <c r="J6" s="1">
-        <v>6468</v>
-      </c>
-      <c r="K6" s="1">
-        <v>7910</v>
-      </c>
-      <c r="L6" s="1">
-        <v>4638</v>
-      </c>
-      <c r="M6" s="1">
-        <v>6611</v>
-      </c>
-      <c r="N6" s="1">
-        <v>69707</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19">
+        <v>400</v>
+      </c>
+      <c r="D19">
+        <v>950</v>
+      </c>
+      <c r="E19">
+        <v>843</v>
+      </c>
+      <c r="F19">
+        <v>693</v>
+      </c>
+      <c r="G19">
+        <v>567</v>
+      </c>
+      <c r="H19">
+        <v>497</v>
+      </c>
+      <c r="I19">
+        <v>592</v>
+      </c>
+      <c r="J19">
+        <v>798</v>
+      </c>
+      <c r="K19">
+        <v>911</v>
+      </c>
+      <c r="L19">
+        <v>777</v>
+      </c>
+      <c r="M19" s="1">
+        <v>1517</v>
+      </c>
+      <c r="N19" s="1">
+        <v>1094</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A20">
         <v>19</v>
       </c>
-      <c r="B7" s="1">
-        <v>2725</v>
-      </c>
-      <c r="C7" s="1">
-        <v>2405</v>
-      </c>
-      <c r="D7" s="1">
-        <v>4588</v>
-      </c>
-      <c r="E7" s="1">
-        <v>2817</v>
-      </c>
-      <c r="F7" s="1">
-        <v>3410</v>
-      </c>
-      <c r="G7" s="1">
-        <v>3769</v>
-      </c>
-      <c r="H7" s="1">
-        <v>2890</v>
-      </c>
-      <c r="I7" s="1">
-        <v>3259</v>
-      </c>
-      <c r="J7" s="1">
-        <v>3373</v>
-      </c>
-      <c r="K7" s="1">
-        <v>5372</v>
-      </c>
-      <c r="L7" s="1">
-        <v>4465</v>
-      </c>
-      <c r="M7" s="1">
-        <v>4747</v>
-      </c>
-      <c r="N7" s="1">
-        <v>43820</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20">
+        <v>724</v>
+      </c>
+      <c r="D20" s="1">
+        <v>1034</v>
+      </c>
+      <c r="E20">
+        <v>874</v>
+      </c>
+      <c r="F20">
+        <v>801</v>
+      </c>
+      <c r="G20">
+        <v>495</v>
+      </c>
+      <c r="H20">
+        <v>387</v>
+      </c>
+      <c r="I20">
+        <v>711</v>
+      </c>
+      <c r="J20">
+        <v>754</v>
+      </c>
+      <c r="K20">
+        <v>591</v>
+      </c>
+      <c r="L20">
+        <v>766</v>
+      </c>
+      <c r="M20">
+        <v>772</v>
+      </c>
+      <c r="N20" s="1">
+        <v>1062</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>20</v>
       </c>
-      <c r="B8" s="1">
-        <v>2322</v>
-      </c>
-      <c r="C8" s="1">
-        <v>4159</v>
-      </c>
-      <c r="D8" s="1">
-        <v>4587</v>
-      </c>
-      <c r="E8" s="1">
-        <v>2674</v>
-      </c>
-      <c r="F8" s="1">
-        <v>3032</v>
-      </c>
-      <c r="G8" s="1">
-        <v>2421</v>
-      </c>
-      <c r="H8" s="1">
-        <v>2404</v>
-      </c>
-      <c r="I8" s="1">
-        <v>3854</v>
-      </c>
-      <c r="J8" s="1">
-        <v>3150</v>
-      </c>
-      <c r="K8" s="1">
-        <v>4322</v>
-      </c>
-      <c r="L8" s="1">
-        <v>3940</v>
-      </c>
-      <c r="M8" s="1">
-        <v>3751</v>
-      </c>
-      <c r="N8" s="1">
-        <v>40616</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="1">
-        <v>2273</v>
-      </c>
-      <c r="C9" s="1">
-        <v>4684</v>
-      </c>
-      <c r="D9" s="1">
-        <v>4746</v>
-      </c>
-      <c r="E9" s="1">
-        <v>1739</v>
-      </c>
-      <c r="F9" s="1">
-        <v>1275</v>
-      </c>
-      <c r="G9" s="1">
-        <v>1194</v>
-      </c>
-      <c r="H9" s="1">
-        <v>1483</v>
-      </c>
-      <c r="I9" s="1">
-        <v>2134</v>
-      </c>
-      <c r="J9" s="1">
-        <v>2316</v>
-      </c>
-      <c r="K9" s="1">
-        <v>2499</v>
-      </c>
-      <c r="L9" s="1">
-        <v>3710</v>
-      </c>
-      <c r="M9" s="1">
-        <v>4393</v>
-      </c>
-      <c r="N9" s="1">
-        <v>32446</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="1">
-        <v>1502</v>
-      </c>
-      <c r="C10" s="1">
-        <v>2448</v>
-      </c>
-      <c r="D10" s="1">
-        <v>2720</v>
-      </c>
-      <c r="E10" s="1">
-        <v>2095</v>
-      </c>
-      <c r="F10" s="1">
-        <v>1797</v>
-      </c>
-      <c r="G10" s="1">
-        <v>1923</v>
-      </c>
-      <c r="H10" s="1">
-        <v>2185</v>
-      </c>
-      <c r="I10" s="1">
-        <v>2705</v>
-      </c>
-      <c r="J10" s="1">
-        <v>2393</v>
-      </c>
-      <c r="K10" s="1">
-        <v>2313</v>
-      </c>
-      <c r="L10" s="1">
-        <v>2632</v>
-      </c>
-      <c r="M10" s="1">
-        <v>2482</v>
-      </c>
-      <c r="N10" s="1">
-        <v>27195</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="1">
-        <v>2080</v>
-      </c>
-      <c r="C11" s="1">
-        <v>3337</v>
-      </c>
-      <c r="D11" s="1">
-        <v>2797</v>
-      </c>
-      <c r="E11" s="1">
-        <v>1455</v>
-      </c>
-      <c r="F11" s="1">
-        <v>1367</v>
-      </c>
-      <c r="G11" s="1">
-        <v>1162</v>
-      </c>
-      <c r="H11" s="1">
-        <v>1385</v>
-      </c>
-      <c r="I11" s="1">
-        <v>1527</v>
-      </c>
-      <c r="J11" s="1">
-        <v>1937</v>
-      </c>
-      <c r="K11" s="1">
-        <v>1986</v>
-      </c>
-      <c r="L11" s="1">
-        <v>2243</v>
-      </c>
-      <c r="M11" s="1">
-        <v>2669</v>
-      </c>
-      <c r="N11" s="1">
-        <v>23945</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="1">
-        <v>1256</v>
-      </c>
-      <c r="C12" s="1">
-        <v>3305</v>
-      </c>
-      <c r="D12" s="1">
-        <v>3322</v>
-      </c>
-      <c r="E12" s="1">
-        <v>1487</v>
-      </c>
-      <c r="F12" s="1">
-        <v>1147</v>
-      </c>
-      <c r="G12">
-        <v>783</v>
-      </c>
-      <c r="H12" s="1">
-        <v>1568</v>
-      </c>
-      <c r="I12" s="1">
-        <v>1746</v>
-      </c>
-      <c r="J12" s="1">
-        <v>1767</v>
-      </c>
-      <c r="K12" s="1">
-        <v>2339</v>
-      </c>
-      <c r="L12" s="1">
-        <v>2340</v>
-      </c>
-      <c r="M12" s="1">
-        <v>2286</v>
-      </c>
-      <c r="N12" s="1">
-        <v>23346</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="1">
-        <v>1389</v>
-      </c>
-      <c r="C13" s="1">
-        <v>2018</v>
-      </c>
-      <c r="D13" s="1">
-        <v>2096</v>
-      </c>
-      <c r="E13" s="1">
-        <v>1193</v>
-      </c>
-      <c r="F13" s="1">
-        <v>1010</v>
-      </c>
-      <c r="G13">
-        <v>755</v>
-      </c>
-      <c r="H13" s="1">
-        <v>1265</v>
-      </c>
-      <c r="I13" s="1">
-        <v>1852</v>
-      </c>
-      <c r="J13" s="1">
-        <v>1078</v>
-      </c>
-      <c r="K13" s="1">
-        <v>1120</v>
-      </c>
-      <c r="L13" s="1">
-        <v>1549</v>
-      </c>
-      <c r="M13" s="1">
-        <v>2037</v>
-      </c>
-      <c r="N13" s="1">
-        <v>17362</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14">
-        <v>764</v>
-      </c>
-      <c r="C14" s="1">
-        <v>2382</v>
-      </c>
-      <c r="D14" s="1">
-        <v>1828</v>
-      </c>
-      <c r="E14" s="1">
-        <v>1019</v>
-      </c>
-      <c r="F14">
-        <v>559</v>
-      </c>
-      <c r="G14">
-        <v>580</v>
-      </c>
-      <c r="H14">
-        <v>814</v>
-      </c>
-      <c r="I14" s="1">
-        <v>2399</v>
-      </c>
-      <c r="J14" s="1">
-        <v>1252</v>
-      </c>
-      <c r="K14" s="1">
-        <v>1103</v>
-      </c>
-      <c r="L14" s="1">
-        <v>1804</v>
-      </c>
-      <c r="M14" s="1">
-        <v>2602</v>
-      </c>
-      <c r="N14" s="1">
-        <v>17106</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="1">
-        <v>2322</v>
-      </c>
-      <c r="C15" s="1">
-        <v>2776</v>
-      </c>
-      <c r="D15" s="1">
-        <v>2537</v>
-      </c>
-      <c r="E15">
-        <v>975</v>
-      </c>
-      <c r="F15">
-        <v>709</v>
-      </c>
-      <c r="G15">
-        <v>470</v>
-      </c>
-      <c r="H15">
-        <v>685</v>
-      </c>
-      <c r="I15">
-        <v>794</v>
-      </c>
-      <c r="J15">
-        <v>717</v>
-      </c>
-      <c r="K15">
-        <v>929</v>
-      </c>
-      <c r="L15" s="1">
-        <v>1338</v>
-      </c>
-      <c r="M15" s="1">
-        <v>1510</v>
-      </c>
-      <c r="N15" s="1">
-        <v>15762</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16">
-        <v>442</v>
-      </c>
-      <c r="C16" s="1">
-        <v>1460</v>
-      </c>
-      <c r="D16" s="1">
-        <v>1530</v>
-      </c>
-      <c r="E16" s="1">
-        <v>1116</v>
-      </c>
-      <c r="F16">
-        <v>652</v>
-      </c>
-      <c r="G16">
-        <v>786</v>
-      </c>
-      <c r="H16">
-        <v>527</v>
-      </c>
-      <c r="I16" s="1">
-        <v>1000</v>
-      </c>
-      <c r="J16" s="1">
-        <v>1453</v>
-      </c>
-      <c r="K16" s="1">
-        <v>1330</v>
-      </c>
-      <c r="L16" s="1">
-        <v>1098</v>
-      </c>
-      <c r="M16" s="1">
-        <v>1057</v>
-      </c>
-      <c r="N16" s="1">
-        <v>12451</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="1">
-        <v>3933</v>
-      </c>
-      <c r="C17" s="1">
-        <v>2542</v>
-      </c>
-      <c r="D17" s="1">
-        <v>2164</v>
-      </c>
-      <c r="E17">
-        <v>308</v>
-      </c>
-      <c r="F17">
-        <v>483</v>
-      </c>
-      <c r="G17">
-        <v>137</v>
-      </c>
-      <c r="H17">
-        <v>220</v>
-      </c>
-      <c r="I17">
-        <v>233</v>
-      </c>
-      <c r="J17">
-        <v>400</v>
-      </c>
-      <c r="K17">
-        <v>365</v>
-      </c>
-      <c r="L17">
-        <v>498</v>
-      </c>
-      <c r="M17">
-        <v>751</v>
-      </c>
-      <c r="N17" s="1">
-        <v>12034</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18">
-        <v>714</v>
-      </c>
-      <c r="C18" s="1">
-        <v>1308</v>
-      </c>
-      <c r="D18" s="1">
-        <v>1100</v>
-      </c>
-      <c r="E18">
-        <v>650</v>
-      </c>
-      <c r="F18">
-        <v>560</v>
-      </c>
-      <c r="G18">
-        <v>555</v>
-      </c>
-      <c r="H18">
-        <v>966</v>
-      </c>
-      <c r="I18">
-        <v>931</v>
-      </c>
-      <c r="J18">
-        <v>894</v>
-      </c>
-      <c r="K18" s="1">
-        <v>1049</v>
-      </c>
-      <c r="L18" s="1">
-        <v>1157</v>
-      </c>
-      <c r="M18" s="1">
-        <v>1321</v>
-      </c>
-      <c r="N18" s="1">
-        <v>11205</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19">
-        <v>400</v>
-      </c>
-      <c r="C19">
-        <v>950</v>
-      </c>
-      <c r="D19">
-        <v>843</v>
-      </c>
-      <c r="E19">
-        <v>693</v>
-      </c>
-      <c r="F19">
-        <v>567</v>
-      </c>
-      <c r="G19">
-        <v>497</v>
-      </c>
-      <c r="H19">
-        <v>592</v>
-      </c>
-      <c r="I19">
-        <v>798</v>
-      </c>
-      <c r="J19">
-        <v>911</v>
-      </c>
-      <c r="K19">
-        <v>777</v>
-      </c>
-      <c r="L19" s="1">
-        <v>1517</v>
-      </c>
-      <c r="M19" s="1">
-        <v>1094</v>
-      </c>
-      <c r="N19" s="1">
-        <v>9639</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20">
-        <v>724</v>
-      </c>
-      <c r="C20" s="1">
-        <v>1034</v>
-      </c>
-      <c r="D20">
-        <v>874</v>
-      </c>
-      <c r="E20">
-        <v>801</v>
-      </c>
-      <c r="F20">
-        <v>495</v>
-      </c>
-      <c r="G20">
-        <v>387</v>
-      </c>
-      <c r="H20">
-        <v>711</v>
-      </c>
-      <c r="I20">
-        <v>754</v>
-      </c>
-      <c r="J20">
-        <v>591</v>
-      </c>
-      <c r="K20">
-        <v>766</v>
-      </c>
-      <c r="L20">
-        <v>772</v>
-      </c>
-      <c r="M20" s="1">
-        <v>1062</v>
-      </c>
-      <c r="N20" s="1">
-        <v>8971</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="1">
+      <c r="B21" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="1">
         <v>1248</v>
       </c>
-      <c r="C21" s="1">
+      <c r="D21" s="1">
         <v>1884</v>
       </c>
-      <c r="D21" s="1">
+      <c r="E21" s="1">
         <v>2111</v>
       </c>
-      <c r="E21">
+      <c r="F21">
         <v>661</v>
       </c>
-      <c r="F21">
+      <c r="G21">
         <v>273</v>
       </c>
-      <c r="G21">
+      <c r="H21">
         <v>126</v>
       </c>
-      <c r="H21">
+      <c r="I21">
         <v>266</v>
       </c>
-      <c r="I21">
+      <c r="J21">
         <v>140</v>
       </c>
-      <c r="J21">
+      <c r="K21">
         <v>185</v>
       </c>
-      <c r="K21">
+      <c r="L21">
         <v>360</v>
       </c>
-      <c r="L21">
+      <c r="M21">
         <v>708</v>
       </c>
-      <c r="M21">
+      <c r="N21">
         <v>978</v>
-      </c>
-      <c r="N21" s="1">
-        <v>8940</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>34</v>
-      </c>
-      <c r="B22" s="1">
-        <v>9335</v>
-      </c>
-      <c r="C22" s="1">
-        <v>19949</v>
-      </c>
-      <c r="D22" s="1">
-        <v>15098</v>
-      </c>
-      <c r="E22" s="1">
-        <v>7559</v>
-      </c>
-      <c r="F22" s="1">
-        <v>6300</v>
-      </c>
-      <c r="G22" s="1">
-        <v>5746</v>
-      </c>
-      <c r="H22" s="1">
-        <v>6834</v>
-      </c>
-      <c r="I22" s="1">
-        <v>7324</v>
-      </c>
-      <c r="J22" s="1">
-        <v>9682</v>
-      </c>
-      <c r="K22" s="1">
-        <v>10725</v>
-      </c>
-      <c r="L22" s="1">
-        <v>14629</v>
-      </c>
-      <c r="M22" s="1">
-        <v>15572</v>
-      </c>
-      <c r="N22" s="1">
-        <v>128753</v>
       </c>
     </row>
   </sheetData>
@@ -1590,10 +1540,10 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>41</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1637,7 +1587,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="C2" s="1">
         <v>346778</v>
@@ -1681,7 +1631,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C3" s="1">
         <v>226458</v>
@@ -1725,7 +1675,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="C4" s="1">
         <v>64967</v>
@@ -1769,7 +1719,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="C5" s="1">
         <v>58012</v>
@@ -1813,7 +1763,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1">
         <v>58670</v>
@@ -1857,7 +1807,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>19</v>
       </c>
       <c r="C7" s="1">
         <v>45647</v>
@@ -1901,7 +1851,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="C8" s="1">
         <v>50924</v>
@@ -1945,7 +1895,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="C9" s="1">
         <v>34046</v>
@@ -1989,7 +1939,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="C10" s="1">
         <v>25668</v>
@@ -2033,7 +1983,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="C11" s="1">
         <v>23510</v>
@@ -2077,7 +2027,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="C12" s="1">
         <v>19773</v>
@@ -2121,7 +2071,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="C13" s="1">
         <v>24282</v>
@@ -2165,7 +2115,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="C14" s="1">
         <v>12094</v>
@@ -2209,7 +2159,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="C15" s="1">
         <v>12493</v>
@@ -2253,7 +2203,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="C16" s="1">
         <v>8678</v>
@@ -2297,7 +2247,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="C17" s="1">
         <v>8256</v>
@@ -2341,7 +2291,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C18" s="1">
         <v>9941</v>
@@ -2385,7 +2335,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="C19" s="1">
         <v>12240</v>
@@ -2429,7 +2379,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="C20" s="1">
         <v>10821</v>
@@ -2473,7 +2423,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
       <c r="C21" s="1">
         <v>6951</v>
@@ -2517,7 +2467,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="C22" s="1">
         <v>3068</v>
@@ -2561,7 +2511,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="C23" s="1">
         <v>2537</v>
@@ -2602,7 +2552,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="C24" s="1">
         <v>2092</v>
@@ -2646,7 +2596,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="C25" s="1">
         <v>1088</v>
@@ -2690,7 +2640,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="C26">
         <v>984</v>
@@ -2734,7 +2684,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>61</v>
+        <v>39</v>
       </c>
       <c r="C27">
         <v>936</v>
@@ -2778,7 +2728,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>62</v>
+        <v>40</v>
       </c>
       <c r="C28" s="1">
         <v>829368</v>

</xml_diff>